<commit_message>
Update DANTON TAR 1/I (TK II) to IPDA Andi Dwi Susilo, S.Kom
NRP 88101015, replacing the previous officer on record for Peleton 1
Kompi I Tingkat II.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA_DANTON_DANKI.xlsx
+++ b/DATA_DANTON_DANKI.xlsx
@@ -649,12 +649,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>RAHMAT HERSA WIDIATMOKO, S.Tr.K.</t>
+          <t>ANDI DWI SUSILO, S.Kom</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>IPTU</t>
+          <t>IPDA</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>01111489</t>
+          <t>88101015</t>
         </is>
       </c>
     </row>

</xml_diff>